<commit_message>
Metal: washers under the back motor screws; duplicate-component check
- Metal back corners: two M3 washers under each M3 x 35 motor screw head,
  so 3.68 mm of thread goes into the motor (was 4.88). Build note added to
  the Metal README and the landing page; BOM washer row is now 24.
- M3 washer renamed to "M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)" in the
  CF and Metal assemblies and BOMs.
- Copy-pasted components (Fusion "Name (1)") replaced with instances in the
  CF and Metal XY joints and the Metal back right; no geometry changes.
- tools/step_bom.py: new "dupes" mode, also run by "check", that flags
  copy-pasted components in the main and every sub-assembly (stock Sovol
  Z carriage parts are listed but not failed). Fixed wrapped STEP names
  picking up a stray space.
- Regenerated CF and Metal STLs, renders and the landing image.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Metal Version/SV08_M5_BOM_from_STEP.xlsx
+++ b/Metal Version/SV08_M5_BOM_from_STEP.xlsx
@@ -1097,11 +1097,11 @@
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>M3 Washer (3mm ID | 7mm OD | .5mm Tall)</t>
+          <t>M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1109,7 +1109,11 @@
           <t>https://amazon.com/dp/B0C3TJ7PWT</t>
         </is>
       </c>
-      <c r="E33" s="2" t="n"/>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>8 for the XY joints, plus 2 under the head of each back motor screw (16) so the M3 x 35 screws don't bottom out in the motor. Or skip those 16 and trim 1-2 mm off each back motor screw.</t>
+        </is>
+      </c>
     </row>
     <row r="34" s="6">
       <c r="A34" s="2" t="inlineStr">

</xml_diff>

<commit_message>
BOMs: break out the linear rail mounting screws and M3 T-nuts into their own section
step_bom category_by_assembly accepts {as, only} to move only matching parts of a group.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Metal Version/SV08_M5_BOM_from_STEP.xlsx
+++ b/Metal Version/SV08_M5_BOM_from_STEP.xlsx
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E93"/>
+  <dimension ref="A1:E94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="6" min="1" max="1"/>
@@ -552,19 +552,15 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>M3 x 8mm SHCS</t>
+          <t>M4 x 10mm BHCS</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0F5Q6YYWM</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>Count matches the 28 M3 T-Nuts 1:1.</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B0CTH3Z2F5</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
     </row>
     <row r="7" s="6">
       <c r="A7" s="2" t="inlineStr">
@@ -573,19 +569,23 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>M4 x 10mm BHCS</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0CTH3Z2F5</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
+          <t>M3 x 5mm FHCS</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B07WFF95JS</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Bearing retainers: 4 per XY joint and 4 per front bottom plate. They end flush with the 5mm plate. Use threadlocker (blue).</t>
+        </is>
+      </c>
     </row>
     <row r="8" s="6">
       <c r="A8" s="2" t="inlineStr">
@@ -594,21 +594,21 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>M3 x 5mm FHCS</t>
+          <t>M3 x 4mm FHCS</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B07WFF95JS</t>
+          <t>https://www.mcmaster.com/92125A127/</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Bearing retainers: 4 per XY joint and 4 per front bottom plate. They end flush with the 5mm plate. Use threadlocker (blue).</t>
+          <t>Bearing retainers: 2 per back top plate (they end on the floor of the pulley-clearance relief) and 2 per front top plate. McMaster-Carr 92125A127 or any M3 x 4mm flat head. Use threadlocker (blue).</t>
         </is>
       </c>
     </row>
@@ -619,23 +619,19 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>M3 x 4mm FHCS</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>https://www.mcmaster.com/92125A127/</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Bearing retainers: 2 per back top plate (they end on the floor of the pulley-clearance relief) and 2 per front top plate. McMaster-Carr 92125A127 or any M3 x 4mm flat head. Use threadlocker (blue).</t>
-        </is>
-      </c>
+          <t>M3 x 10mm BHCS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0GJK7Z9DH</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
     </row>
     <row r="10" s="6">
       <c r="A10" s="2" t="inlineStr">
@@ -644,16 +640,16 @@
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>M3 x 10mm BHCS</t>
+          <t>M3 x 35mm SHCS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0GJK7Z9DH</t>
+          <t>https://amazon.com/dp/B0GHY9ZCLC</t>
         </is>
       </c>
       <c r="E10" s="2" t="n"/>
@@ -669,12 +665,12 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>M3 x 35mm SHCS</t>
+          <t>M4 x 45mm BHCS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0GHY9ZCLC</t>
+          <t>https://amazon.com/dp/B0GH6G1R1G</t>
         </is>
       </c>
       <c r="E11" s="2" t="n"/>
@@ -690,15 +686,19 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>M4 x 45mm BHCS</t>
+          <t>M3 x 10mm Ultra Thin Flat Head (.8-1mm)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0GH6G1R1G</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
+          <t>https://amazon.com/dp/B0H61WCTBX</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ultra-thin head (.8-1mm). 2 per front motor assembly and 2 per XY joint. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
+        </is>
+      </c>
     </row>
     <row r="13" s="6">
       <c r="A13" s="2" t="inlineStr">
@@ -707,21 +707,21 @@
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>M3 x 10mm Ultra Thin Flat Head (.8-1mm)</t>
+          <t>M2 x 2mm Set Screw</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0H61WCTBX</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Ultra-thin head (.8-1mm). 2 per front motor assembly and 2 per XY joint. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
+          <t>https://amazon.com/dp/B0DDJBSF6B</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Should come with the GT2 20-Tooth Pulley - Live Idler Version (2 per pulley, 4 total).</t>
         </is>
       </c>
     </row>
@@ -736,17 +736,17 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>M2 x 2mm Set Screw</t>
+          <t>M2 x 8mm SHCS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DDJBSF6B</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Should come with the GT2 20-Tooth Pulley - Live Idler Version (2 per pulley, 4 total).</t>
+          <t>https://amazon.com/dp/B0D4JMPT86</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Endstop screws. They thread straight into tapped M2 holes in the back top plates (no nuts).</t>
         </is>
       </c>
     </row>
@@ -761,19 +761,15 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>M2 x 8mm SHCS</t>
+          <t>M4 x 20mm BHCS</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D4JMPT86</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Endstop screws. They thread straight into tapped M2 holes in the back top plates (no nuts).</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B0DYSQZHC9</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
     </row>
     <row r="16" s="6">
       <c r="A16" s="2" t="inlineStr">
@@ -786,41 +782,45 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>M4 x 20mm BHCS</t>
+          <t>M5 x 45mm BHCS</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DYSQZHC9</t>
+          <t>https://amazon.com/dp/B0GJX8PR8J</t>
         </is>
       </c>
       <c r="E16" s="2" t="n"/>
     </row>
     <row r="17" s="6">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Screws</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>M5 x 45mm BHCS</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0GJX8PR8J</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="n"/>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Fasteners - Shoulder Bolts</t>
+        </is>
+      </c>
     </row>
     <row r="18" s="6">
-      <c r="A18" s="7" t="inlineStr">
-        <is>
-          <t>Fasteners - Shoulder Bolts</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Shoulder Bolts</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>D5 M3 x 30mm Shoulder Bolt</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256810189139611.html</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Make sure you select Size D5-M3, Length 30mm</t>
         </is>
       </c>
     </row>
@@ -831,11 +831,11 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>D5 M3 x 30mm Shoulder Bolt</t>
+          <t>D5 M3 x 25mm Shoulder Bolt</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Make sure you select Size D5-M3, Length 30mm</t>
+          <t>Make sure you select Size D5-M3, Length 25mm</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>D5 M3 x 25mm Shoulder Bolt</t>
+          <t>D5 M3 x 35mm Shoulder Bolt</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -870,173 +870,177 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Make sure you select Size D5-M3, Length 25mm</t>
+          <t>Make sure you select Size D5-M3, Length 35mm</t>
         </is>
       </c>
     </row>
     <row r="21" s="6">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Shoulder Bolts</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>D5 M3 x 35mm Shoulder Bolt</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>https://www.aliexpress.us/item/3256810189139611.html</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Make sure you select Size D5-M3, Length 35mm</t>
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Fasteners - T-Nuts</t>
         </is>
       </c>
     </row>
     <row r="22" s="6">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Fasteners - T-Nuts</t>
-        </is>
-      </c>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>T-Nuts</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>M4 T-Nut</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0C9DJBG1H</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
     </row>
     <row r="23" s="6">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>T-Nuts</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>M4 T-Nut</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0C9DJBG1H</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Fasteners - Threaded Rods</t>
+        </is>
+      </c>
     </row>
     <row r="24" s="6">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>T-Nuts</t>
+          <t>Threaded Rods</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>M3 T-Nut</t>
+          <t>M3 Internally Threaded Spacer (5mm OD | 35mm Tall)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0G2M7W3PL</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
+          <t>https://amazon.com/dp/B0D3HWQ2GF</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+        </is>
+      </c>
     </row>
     <row r="25" s="6">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t>Fasteners - Threaded Rods</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Threaded Rods</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>M3 Internally Threaded Spacer (5mm OD | 25mm Tall)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0D3HVVJPN</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
         </is>
       </c>
     </row>
     <row r="26" s="6">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Threaded Rods</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 35mm Tall)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0D3HWQ2GF</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Fasteners - Nuts</t>
         </is>
       </c>
     </row>
     <row r="27" s="6">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Nuts</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 25mm Tall)</t>
+          <t>M5 Nut</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HVVJPN</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B0D1X2YBLJ</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
     </row>
     <row r="28" s="6">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Fasteners - Nuts</t>
+          <t>Washers &amp; Shims</t>
         </is>
       </c>
     </row>
     <row r="29" s="6">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Nuts</t>
+          <t>Washers &amp; Shims</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>M5 Nut</t>
+          <t>M5 Washer (5mm ID | 10mm OD | 1mm Tall)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D1X2YBLJ</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
+          <t>https://amazon.com/dp/B07WZ5WQCG</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Includes the 36 bearing-stack shims, and 2 under each front shoulder-bolt head (16) so the bolts thread 4mm into the motor. Or trim those bolts' threads to 4mm and skip those 16.</t>
+        </is>
+      </c>
     </row>
     <row r="30" s="6">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>Washers &amp; Shims</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>M4 Washer (4mm ID | 9mm OD | 1mm Tall)</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DK6KXB6W</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>.8mm more common and acceptable swap, OD matters</t>
         </is>
       </c>
     </row>
@@ -1047,21 +1051,21 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>M5 Washer (5mm ID | 10mm OD | 1mm Tall)</t>
+          <t>M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B07WZ5WQCG</t>
-        </is>
-      </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>Includes the 36 bearing-stack shims, and 2 under each front shoulder-bolt head (16) so the bolts thread 4mm into the motor. Or trim those bolts' threads to 4mm and skip those 16.</t>
+          <t>https://amazon.com/dp/B0C3TJ7PWT</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>8 for the XY joints, plus 2 under the head of each back motor screw (16) so the M3 x 35 screws don't bottom out in the motor. Or skip those 16 and trim 1-2 mm off each back motor screw.</t>
         </is>
       </c>
     </row>
@@ -1072,229 +1076,229 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>M4 Washer (4mm ID | 9mm OD | 1mm Tall)</t>
+          <t>M3 Shim (3mm ID | 5mm OD | .2mm Tall)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DK6KXB6W</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>.8mm more common and acceptable swap, OD matters</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B08ZYP1TK4</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
     </row>
     <row r="33" s="6">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Washers &amp; Shims</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t>M3 Washer (3mm ID | 7mm OD | .5-.6mm Tall)</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0C3TJ7PWT</t>
-        </is>
-      </c>
-      <c r="E33" s="2" t="inlineStr">
-        <is>
-          <t>8 for the XY joints, plus 2 under the head of each back motor screw (16) so the M3 x 35 screws don't bottom out in the motor. Or skip those 16 and trim 1-2 mm off each back motor screw.</t>
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Bearings</t>
         </is>
       </c>
     </row>
     <row r="34" s="6">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Washers &amp; Shims</t>
+          <t>Bearings</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>8</v>
+        <v>48</v>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>M3 Shim (3mm ID | 5mm OD | .2mm Tall)</t>
+          <t>695-2RS Flanged Bearing</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B08ZYP1TK4</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="n"/>
+          <t>https://amazon.com/dp/B0CGXF48ZZ</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Includes the 12 loose bearings named F695-2RS Bearing Single in CAD (36 stacked + 12 loose).</t>
+        </is>
+      </c>
     </row>
     <row r="35" s="6">
-      <c r="A35" s="7" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Bearings</t>
         </is>
       </c>
+      <c r="B35" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>MR63ZZ Bearing 3x6x2.5mm</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DY11G865</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
     </row>
     <row r="36" s="6">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Bearings</t>
-        </is>
-      </c>
-      <c r="B36" s="3" t="n">
-        <v>48</v>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>695-2RS Flanged Bearing</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0CGXF48ZZ</t>
-        </is>
-      </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>Includes the 12 loose bearings named F695-2RS Bearing Single in CAD (36 stacked + 12 loose).</t>
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Pulleys</t>
         </is>
       </c>
     </row>
     <row r="37" s="6">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Bearings</t>
+          <t>Pulleys</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>MR63ZZ Bearing 3x6x2.5mm</t>
+          <t>GT2 20-Tooth Pulley Set-Screw Version</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0DY11G865</t>
+          <t>https://amazon.com/dp/B0GWLM6FD6</t>
         </is>
       </c>
       <c r="E37" s="2" t="n"/>
     </row>
     <row r="38" s="6">
-      <c r="A38" s="7" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>Pulleys</t>
         </is>
       </c>
+      <c r="B38" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>GT2 20-Tooth Pulley - Live Idler Version</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://www.aliexpress.us/item/3256803833151466.html</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Make sure you select Bore 5mm Width 6mm. Uses 2x M2 x 2mm Set Screws each (4 total). Pulley body recovered from an unnamed STEP node (one per XY Joint)</t>
+        </is>
+      </c>
     </row>
     <row r="39" s="6">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Pulleys</t>
-        </is>
-      </c>
-      <c r="B39" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>GT2 20-Tooth Pulley Set-Screw Version</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0GWLM6FD6</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="n"/>
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Belts</t>
+        </is>
+      </c>
     </row>
     <row r="40" s="6">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>Pulleys</t>
+          <t>Belts</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>GT2 20-Tooth Pulley - Live Idler Version</t>
+          <t>Bottom Belt 2.1m</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.us/item/3256803833151466.html</t>
-        </is>
-      </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>Make sure you select Bore 5mm Width 6mm. Uses 2x M2 x 2mm Set Screws each (4 total). Pulley body recovered from an unnamed STEP node (one per XY Joint)</t>
-        </is>
-      </c>
+          <t>https://amazon.com/dp/B07CDDPCM8</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="n"/>
     </row>
     <row r="41" s="6">
-      <c r="A41" s="7" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Belts</t>
         </is>
       </c>
+      <c r="B41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Top Belt 2.1m</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B07CDDPCM8</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n"/>
     </row>
     <row r="42" s="6">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Belts</t>
-        </is>
-      </c>
-      <c r="B42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>Bottom Belt 2.1m</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B07CDDPCM8</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="n"/>
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Spacers (Aluminum)</t>
+        </is>
+      </c>
     </row>
     <row r="43" s="6">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Belts</t>
+          <t>Spacers (Aluminum)</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Top Belt 2.1m</t>
+          <t>M5 Spacer 10mm OD 10mm Tall</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B07CDDPCM8</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
+          <t>https://www.aliexpress.com/item/3256802878592600.html</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.. If purchasing from Aliexpress be sure to select 5.1x10x10</t>
+        </is>
+      </c>
     </row>
     <row r="44" s="6">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Spacers (Aluminum)</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>M3 Spacer 8mm OD 20mm Tall</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0F8QLBKYC</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
@@ -1305,21 +1309,21 @@
         </is>
       </c>
       <c r="B45" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 10mm OD 10mm Tall</t>
+          <t>M5 Spacer 8mm OD 20mm Tall</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://www.aliexpress.com/item/3256802878592600.html</t>
+          <t>https://amazon.com/dp/B0CRL77N5C</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
         <is>
-          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.. If purchasing from Aliexpress be sure to select 5.1x10x10</t>
+          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
@@ -1330,21 +1334,21 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>M3 Spacer 8mm OD 20mm Tall</t>
+          <t>M5 Spacer 8mm OD 30mm Tall</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0F8QLBKYC</t>
+          <t>https://amazon.com/dp/B0CQ53LS2B</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
@@ -1355,78 +1359,78 @@
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 8mm OD 20mm Tall</t>
+          <t>M5 Spacer 10mm OD 20mm Tall</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0CRL77N5C</t>
+          <t>https://amazon.com/dp/B0D2L3H5LV</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
         <is>
-          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
         </is>
       </c>
     </row>
     <row r="48" s="6">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Spacers (Aluminum)</t>
-        </is>
-      </c>
-      <c r="B48" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>M5 Spacer 8mm OD 30mm Tall</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0CQ53LS2B</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>Purchase preferred. Printed as alternative with same dimensions.</t>
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Xol Toolhead Hardware</t>
         </is>
       </c>
     </row>
     <row r="49" s="6">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>Spacers (Aluminum)</t>
+          <t>Xol Toolhead Hardware</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>M5 Spacer 10mm OD 20mm Tall</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0D2L3H5LV</t>
+          <t>M3 x 6mm BHCS</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="E49" s="4" t="inlineStr">
         <is>
-          <t>8mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
     <row r="50" s="6">
-      <c r="A50" s="7" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Xol Toolhead Hardware</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>M2 x 12mm BHCS</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1437,11 +1441,11 @@
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>M3 x 6mm BHCS</t>
+          <t>M3 x 30mm Dowel Pin</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1451,7 +1455,7 @@
       </c>
       <c r="E51" s="4" t="inlineStr">
         <is>
-          <t>Not required unless building the Xol carriage.</t>
+          <t>Only dowel used by the Xol Toolhead. Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1466,7 +1470,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>M2 x 12mm BHCS</t>
+          <t>Xol 6mm Clamp</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1487,11 +1491,11 @@
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>M3 x 30mm Dowel Pin</t>
+          <t>D2F-L Micro Switch (Endstop)</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1501,7 +1505,7 @@
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Only dowel used by the Xol Toolhead. Not required unless building the Xol carriage.</t>
+          <t>Not required unless building the Xol carriage.</t>
         </is>
       </c>
     </row>
@@ -1512,11 +1516,11 @@
         </is>
       </c>
       <c r="B54" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Xol 6mm Clamp</t>
+          <t>Xol-Carriage_MGN12H_MGN9H_archetype_clips</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -1531,66 +1535,48 @@
       </c>
     </row>
     <row r="55" s="6">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>Xol Toolhead Hardware</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>D2F-L Micro Switch (Endstop)</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>Not required unless building the Xol carriage.</t>
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>Electronics / Endstops</t>
         </is>
       </c>
     </row>
     <row r="56" s="6">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Xol Toolhead Hardware</t>
+          <t>Electronics / Endstops</t>
         </is>
       </c>
       <c r="B56" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Xol-Carriage_MGN12H_MGN9H_archetype_clips</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+          <t>D2F-L Micro Switch (Endstop)</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0DBV8XGG4</t>
         </is>
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
-          <t>Not required unless building the Xol carriage.</t>
+          <t>Base machine endstops (one in each back assembly).</t>
         </is>
       </c>
     </row>
     <row r="57" s="6">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Electronics / Endstops</t>
+          <t>Linear Rails &amp; Sliders</t>
         </is>
       </c>
     </row>
     <row r="58" s="6">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Electronics / Endstops</t>
+          <t>Linear Rails &amp; Sliders</t>
         </is>
       </c>
       <c r="B58" s="3" t="n">
@@ -1598,24 +1584,34 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>D2F-L Micro Switch (Endstop)</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>https://amazon.com/dp/B0DBV8XGG4</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>Base machine endstops (one in each back assembly).</t>
+          <t>MGN9H Linear Rail Slide</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="n"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Re-usable from Stock</t>
         </is>
       </c>
     </row>
     <row r="59" s="6">
-      <c r="A59" s="7" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Linear Rails &amp; Sliders</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Y MGN9H Rail 402mm</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>Re-usable from Stock</t>
         </is>
       </c>
     </row>
@@ -1626,11 +1622,11 @@
         </is>
       </c>
       <c r="B60" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>MGN9H Linear Rail Slide</t>
+          <t>MGN12H Linear Rail Slide</t>
         </is>
       </c>
       <c r="D60" s="2" t="n"/>
@@ -1647,11 +1643,11 @@
         </is>
       </c>
       <c r="B61" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Y MGN9H Rail 402mm</t>
+          <t>X MGN12H Rail 406mm</t>
         </is>
       </c>
       <c r="D61" s="2" t="n"/>
@@ -1662,94 +1658,92 @@
       </c>
     </row>
     <row r="62" s="6">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Linear Rails &amp; Sliders</t>
-        </is>
-      </c>
-      <c r="B62" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>MGN12H Linear Rail Slide</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="n"/>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Re-usable from Stock</t>
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Linear Rail Mounting Hardware</t>
         </is>
       </c>
     </row>
     <row r="63" s="6">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>Linear Rails &amp; Sliders</t>
+          <t>Linear Rail Mounting Hardware</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>X MGN12H Rail 406mm</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="n"/>
+          <t>M3 x 8mm SHCS</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0F5Q6YYWM</t>
+        </is>
+      </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Re-usable from Stock</t>
+          <t>Rail mounting screws: 10 per Y rail (20) and 8 on the X rail, one per M3 T-Nut.</t>
         </is>
       </c>
     </row>
     <row r="64" s="6">
-      <c r="A64" s="7" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Linear Rail Mounting Hardware</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>M3 T-Nut</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://amazon.com/dp/B0G2M7W3PL</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Rail mounting T-nuts: 10 per Y rail (20) and 8 on the X rail.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" s="6">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t>Motors</t>
         </is>
       </c>
     </row>
-    <row r="65" s="6">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="66" s="6">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Motors</t>
         </is>
       </c>
-      <c r="B65" s="3" t="n">
+      <c r="B66" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C65" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>42-48 Motor 5mmx30-37mm Shaft</t>
         </is>
       </c>
-      <c r="D65" s="2" t="n"/>
-      <c r="E65" s="2" t="n"/>
-    </row>
-    <row r="66" s="6">
-      <c r="A66" s="7" t="inlineStr">
+      <c r="D66" s="2" t="n"/>
+      <c r="E66" s="2" t="n"/>
+    </row>
+    <row r="67" s="6">
+      <c r="A67" s="7" t="inlineStr">
         <is>
           <t>Extrusions</t>
         </is>
       </c>
-    </row>
-    <row r="67" s="6">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>Extrusions</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Gantry Y-Axis 2020 Extrusion 469mm</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="n"/>
-      <c r="E67" s="2" t="n"/>
     </row>
     <row r="68" s="6">
       <c r="A68" s="2" t="inlineStr">
@@ -1758,19 +1752,15 @@
         </is>
       </c>
       <c r="B68" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Gantry X-Axis 2020 Extrusion 342mm</t>
+          <t>Gantry Y-Axis 2020 Extrusion 469mm</t>
         </is>
       </c>
       <c r="D68" s="2" t="n"/>
-      <c r="E68" s="4" t="inlineStr">
-        <is>
-          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts.</t>
-        </is>
-      </c>
+      <c r="E68" s="2" t="n"/>
     </row>
     <row r="69" s="6">
       <c r="A69" s="2" t="inlineStr">
@@ -1783,37 +1773,37 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
+          <t>Gantry X-Axis 2020 Extrusion 342mm</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n"/>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" s="6">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Extrusions</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
           <t>Toolhead X-Axis 2020 Extrusion 426mm</t>
         </is>
       </c>
-      <c r="D69" s="2" t="n"/>
-      <c r="E69" s="2" t="n"/>
-    </row>
-    <row r="70" s="6">
-      <c r="A70" s="7" t="inlineStr">
+      <c r="D70" s="2" t="n"/>
+      <c r="E70" s="2" t="n"/>
+    </row>
+    <row r="71" s="6">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t>Metal Plates</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" s="6">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>Metal Plates</t>
-        </is>
-      </c>
-      <c r="B71" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>XY Live Idler Spacer 5mm Metal5mm</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="n"/>
-      <c r="E71" s="4" t="inlineStr">
-        <is>
-          <t>Machined from 5mm 6061 aluminium. See the hole guide in the Metal README.</t>
         </is>
       </c>
     </row>
@@ -1824,11 +1814,11 @@
         </is>
       </c>
       <c r="B72" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Back Left Bottom Plate Metal5mm</t>
+          <t>XY Live Idler Spacer 5mm Metal5mm</t>
         </is>
       </c>
       <c r="D72" s="2" t="n"/>
@@ -1849,7 +1839,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Back Left Top Plate Metal5mm</t>
+          <t>Back Left Bottom Plate Metal5mm</t>
         </is>
       </c>
       <c r="D73" s="2" t="n"/>
@@ -1870,7 +1860,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Back Right Bottom Plate Metal5mm</t>
+          <t>Back Left Top Plate Metal5mm</t>
         </is>
       </c>
       <c r="D74" s="2" t="n"/>
@@ -1891,7 +1881,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Back Right Top Plate Metal5mm</t>
+          <t>Back Right Bottom Plate Metal5mm</t>
         </is>
       </c>
       <c r="D75" s="2" t="n"/>
@@ -1912,7 +1902,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Front Left Bottom Metal5mm</t>
+          <t>Back Right Top Plate Metal5mm</t>
         </is>
       </c>
       <c r="D76" s="2" t="n"/>
@@ -1933,7 +1923,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Front Left Top Metal5mm</t>
+          <t>Front Left Bottom Metal5mm</t>
         </is>
       </c>
       <c r="D77" s="2" t="n"/>
@@ -1954,7 +1944,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Front Right Bottom Metal5mm</t>
+          <t>Front Left Top Metal5mm</t>
         </is>
       </c>
       <c r="D78" s="2" t="n"/>
@@ -1975,7 +1965,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>Front Right Top Metal5mm</t>
+          <t>Front Right Bottom Metal5mm</t>
         </is>
       </c>
       <c r="D79" s="2" t="n"/>
@@ -1996,7 +1986,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Left Bottom Plate Metal5mm</t>
+          <t>Front Right Top Metal5mm</t>
         </is>
       </c>
       <c r="D80" s="2" t="n"/>
@@ -2017,7 +2007,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Left Top Plate Metal5mm</t>
+          <t>XY Live Idler Left Bottom Plate Metal5mm</t>
         </is>
       </c>
       <c r="D81" s="2" t="n"/>
@@ -2038,7 +2028,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Right Bottom Plate Metal5mm</t>
+          <t>XY Live Idler Left Top Plate Metal5mm</t>
         </is>
       </c>
       <c r="D82" s="2" t="n"/>
@@ -2059,7 +2049,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Right Top Plate Metal5mm</t>
+          <t>XY Live Idler Right Bottom Plate Metal5mm</t>
         </is>
       </c>
       <c r="D83" s="2" t="n"/>
@@ -2076,45 +2066,45 @@
         </is>
       </c>
       <c r="B84" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>Tensioner Lever Arm Revised - 5mm Metal Only</t>
+          <t>XY Live Idler Right Top Plate Metal5mm</t>
         </is>
       </c>
       <c r="D84" s="2" t="n"/>
       <c r="E84" s="4" t="inlineStr">
         <is>
+          <t>Machined from 5mm 6061 aluminium. See the hole guide in the Metal README.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" s="6">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Metal Plates</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Tensioner Lever Arm Revised - 5mm Metal Only</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n"/>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
           <t>Flat 5mm metal version of the tensioner lever, machined with the plates. Replaces the shared printed/CF lever. Takes an MR63ZZ bearing in a 6mm H7 seat.</t>
         </is>
       </c>
     </row>
-    <row r="85" s="6">
-      <c r="A85" s="7" t="inlineStr">
+    <row r="86" s="6">
+      <c r="A86" s="7" t="inlineStr">
         <is>
           <t>Printed Parts</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" s="6">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>Printed Parts</t>
-        </is>
-      </c>
-      <c r="B86" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>Z Carriage Spacer</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="n"/>
-      <c r="E86" s="4" t="inlineStr">
-        <is>
-          <t>Check Repo</t>
         </is>
       </c>
     </row>
@@ -2125,11 +2115,11 @@
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Back Spacer Plate 20mm</t>
+          <t>Z Carriage Spacer</t>
         </is>
       </c>
       <c r="D87" s="2" t="n"/>
@@ -2150,7 +2140,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Front Spacer Plate 20mm</t>
+          <t>Back Spacer Plate 20mm</t>
         </is>
       </c>
       <c r="D88" s="2" t="n"/>
@@ -2171,7 +2161,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Printed Back Motor Spacer</t>
+          <t>Front Spacer Plate 20mm</t>
         </is>
       </c>
       <c r="D89" s="2" t="n"/>
@@ -2192,7 +2182,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>XY Live Idler Spacer</t>
+          <t>Printed Back Motor Spacer</t>
         </is>
       </c>
       <c r="D90" s="2" t="n"/>
@@ -2203,11 +2193,25 @@
       </c>
     </row>
     <row r="91" s="6">
-      <c r="A91" s="2" t="n"/>
-      <c r="B91" s="3" t="n"/>
-      <c r="C91" s="2" t="n"/>
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Printed Parts</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>XY Live Idler Spacer</t>
+        </is>
+      </c>
       <c r="D91" s="2" t="n"/>
-      <c r="E91" s="4" t="n"/>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>Check Repo</t>
+        </is>
+      </c>
     </row>
     <row r="92" s="6">
       <c r="A92" s="2" t="n"/>
@@ -2223,27 +2227,35 @@
       <c r="D93" s="2" t="n"/>
       <c r="E93" s="4" t="n"/>
     </row>
+    <row r="94" s="6">
+      <c r="A94" s="2" t="n"/>
+      <c r="B94" s="3" t="n"/>
+      <c r="C94" s="2" t="n"/>
+      <c r="D94" s="2" t="n"/>
+      <c r="E94" s="4" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A64:E64"/>
+  <mergeCells count="20">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A48:E48"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A70:E70"/>
-    <mergeCell ref="A25:E25"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A66:E66"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A65:E65"/>
+    <mergeCell ref="A21:E21"/>
+    <mergeCell ref="A55:E55"/>
+    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A57:E57"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A85:E85"/>
+    <mergeCell ref="A86:E86"/>
+    <mergeCell ref="A42:E42"/>
+    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A71:E71"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A22:E22"/>
-    <mergeCell ref="A35:E35"/>
-    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A17:E17"/>
+    <mergeCell ref="A62:E62"/>
     <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A44:E44"/>
+    <mergeCell ref="A67:E67"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Metal: Chicago bolt live idler shafts, XY holes match the stock toolhead extrusion, metal printed parts 3MF
Metal XY joints and fronts use the M5x40/M5x30 Chicago bolt bases with M4x8 ultra-thin heads.
XY span 40 mm exact; front span 29 mm, so one M5 washer under each front base head (BOM 60 -> 62
washers) and a note to sand the front screw heads to ~1.0 mm (0.2 -> 0.4 mm under the motor).
XY M4 holes now 5 / 25 mm from the stock toolhead extrusion ends: all three versions fit the
stock extrusions. Metal BOM Live Idler Shafts section, stock toolhead note; README build notes;
root README now describes Chicago bolts and stock extrusions for every version; note that
machined aluminium lever arms will be available. New Metal Printed Components.3mf, STL
previews, renders.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Metal Version/SV08_M5_BOM_from_STEP.xlsx
+++ b/Metal Version/SV08_M5_BOM_from_STEP.xlsx
@@ -682,21 +682,21 @@
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>M3 x 10mm Ultra Thin Flat Head (.8-1mm)</t>
+          <t>M4x8 Ultra Thin Flat Head</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0H61WCTBX</t>
+          <t>https://amazon.com/dp/B0H61X7SWB</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Ultra-thin head (.8-1mm). 2 per front motor assembly and 2 per XY joint. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
+          <t>Screw end of each Chicago bolt live idler shaft (1 per front motor assembly and 1 per XY joint). 1.2mm head. METAL: on the 2 at the front corners, sand the head down to about 1.0mm (rub it flat on sandpaper on a flat surface): with the 5mm plates it sits only 0.2mm under the motor as supplied, 0.4mm after sanding. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage the bearings.</t>
         </is>
       </c>
     </row>
@@ -905,14 +905,14 @@
     <row r="23" s="6">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>Fasteners - Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
     </row>
     <row r="24" s="6">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -920,24 +920,24 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 35mm Tall)</t>
+          <t>M5x40 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HWQ2GF</t>
+          <t>https://amazon.com/dp/B0FLJNY14R</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the XY joints (1 per joint). 304 stainless Chicago screw: the 5mm x 40mm barrel runs the full width of both bearings, its head on one bearing and an M4x8 Ultra Thin Flat Head on the other, so the bearings are clamped and the idler can't float. Pack of 20. The M4x4 screws in the pack aren't used: their 2mm heads don't clear the front motors, so the ultra-thin heads are used everywhere. ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 35mm (amazon.com/dp/B0D3HWQ2GF), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 40mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
     <row r="25" s="6">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -945,17 +945,17 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 25mm Tall)</t>
+          <t>M5x30 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HVVJPN</t>
+          <t>https://amazon.com/dp/B0FLJQP39V</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the front motor assemblies (1 per side). 304 stainless Chicago screw: the 5mm x 30mm barrel runs the full width of both bearings, head at the bottom and an M4x8 Ultra Thin Flat Head at the top. METAL: the 5mm plates give a 29mm bearing span, so put one M5 washer (1mm) under the base head as a shim so it clamps the lower bearing, and sand the ultra-thin head down to about 1.0mm (see that row): as supplied it sits only 0.2mm under the motor. Pack of 20; the M4x4 screws in the pack aren't used (their 2mm heads don't clear the motor). ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 25mm (amazon.com/dp/B0D3HVVJPN), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 30mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Includes the 36 bearing-stack shims, and 2 under each front shoulder-bolt head (16) so the bolts thread 4mm into the motor. Or trim those bolts' threads to 4mm and skip those 16.</t>
+          <t>Includes the 36 bearing-stack shims, and 2 under each front shoulder-bolt head (16) so the bolts thread 4mm into the motor. Or trim those bolts' threads to 4mm and skip those 16. Plus 1 under the base head of each front Chicago bolt (2) as a shim: the metal front bearing span is 29mm, 1mm shorter than the bolt. The bearing's inner race stands slightly proud of its seal, so a standard 10mm washer clears the seal.</t>
         </is>
       </c>
     </row>
@@ -1804,7 +1804,7 @@
       <c r="D70" s="2" t="n"/>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>The XY joints don't line up with the stock extrusion's holes (different bolt pattern). Either mount them with M4 T-nuts in the slots, or replace this extrusion with one drilled to match.</t>
+          <t>Stock extrusion works: the XY joint bolt holes line up with its existing holes (5mm and 25mm from each end).</t>
         </is>
       </c>
     </row>

</xml_diff>